<commit_message>
[EXECUTOR] F3 RENUMBER Case_02: U.C.x flattened → UC-01..36 (compliance 01..15 + product 16..36), two-phase, 12 files, 6 SVGs re-rendered, xlsx regenerated; gates: pre-existing FAILs only, audit 100%, mermaid 192/192, smoke 16/16; 1 missed live ref (Doc23) re-anchored
</commit_message>
<xml_diff>
--- a/02_CASES/Case_02_SecureBorder_Solutions/03_PHASE3_DECOMPOSITION/22_Traceability_Matrix_rich_v0.xlsx
+++ b/02_CASES/Case_02_SecureBorder_Solutions/03_PHASE3_DECOMPOSITION/22_Traceability_Matrix_rich_v0.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-04 20:57</t>
+          <t>2026-09-06 00:38</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Doc21_Use_Cases_Catalog.md (mixed U.C.*/UC-* id space)</t>
+          <t>Doc21_Use_Cases_Catalog.md (flat UC-01..UC-36 id space, RENUMBER 2026-09-05)</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>77</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF (no PF 1.0 analogue for product patch/OTA update management)</t>
+          <t>ALT-ANCHOR (SSDF PS.1; 800-53r5 SI-2) (no PF 1.0 analogue for product patch/OTA update management)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF (no PF 1.0 MFA subcategory)</t>
+          <t>ALT-ANCHOR (800-53r5 IA-2(1); ASVS V3.3) (no PF 1.0 MFA subcategory)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1936,12 +1936,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF (no PF 1.0 backup/DR recovery subcategory; CSF IDs corrected to CSF column per Doc19 §1)</t>
+          <t>ALT-ANCHOR (800-53r5 CP-9; CP-10) (no PF 1.0 backup/DR recovery subcategory; CSF IDs corrected to CSF column per Doc19 §1)</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF</t>
+          <t>ALT-ANCHOR (800-53r5 CP-9; CP-10)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF (no PF 1.0 analogue for physical third-party boundary isolation)</t>
+          <t>ALT-ANCHOR (800-53r5 PE-3; PE-6) (no PF 1.0 analogue for physical third-party boundary isolation)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF (no PF 1.0 secure-SDLC subcategory)</t>
+          <t>ALT-ANCHOR (SSDF PW.1; 800-53r5 SA-8) (no PF 1.0 secure-SDLC subcategory)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF (no PF 1.0 board-training subcategory)</t>
+          <t>ALT-ANCHOR (SAMM G-EG-A-1; 800-53r5 AT-2) (no PF 1.0 board-training subcategory)</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3476,12 +3476,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF (no PF 1.0 compliance-testing subcategory; CSF IDs corrected to CSF column per Doc19 §1)</t>
+          <t>ALT-ANCHOR (800-53r5 CA-2; CA-7) (no PF 1.0 compliance-testing subcategory; CSF IDs corrected to CSF column per Doc19 §1)</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>UNMAPPED_PF</t>
+          <t>ALT-ANCHOR (800-53r5 CA-2; CA-7)</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -5262,10 +5262,10 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5321,7 +5321,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>U.C.3.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5356,7 +5356,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5391,7 +5391,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>100% of captured biometric templates pass encryption-validation test (cryptographic nonce decrypted with the expected subject key) within 30s of capture; failure rate &lt; 0.001% across 10,000 captures.</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>100% of raw facial images are unrecoverable from primary storage 60s after template extraction, verified by storage forensics scan; 0 bytes of raw image remain in any store.</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>U.C.3.4.1</t>
+          <t>UC-06</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5496,7 +5496,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>U.C.3.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>U.C.3.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>U.C.3.4.1, U.C.3.6.1</t>
+          <t>UC-06</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -5601,7 +5601,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>U.C.3.5.1</t>
+          <t>UC-07</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>0 default passwords and 0 enabled unused ports on 100% of shipped kiosks, verified by automated config-audit script running on each kiosk image before shipment.</t>
         </is>
       </c>
     </row>
@@ -5636,7 +5636,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5706,7 +5706,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>Sessions terminate in ≤ 15 min (mean) and ≤ 15 min 30s (p99) of inactivity across 1,000 measured idle sessions; no session persists beyond 16 min.</t>
         </is>
       </c>
     </row>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>U.C.3.7.1</t>
+          <t>UC-08</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5756,7 +5756,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>Every AI-decision override produces a justification payload (operator id, reason code, free text) within 30s; 0 overrides accepted without justification in audit log over a 90-day measurement window.</t>
         </is>
       </c>
     </row>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>U.C.1.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>U.C.1.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>U.C.1.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>U.C.1.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5916,7 +5916,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>U.C.1.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>U.C.1.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5986,7 +5986,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>U.C.1.3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>U.C.1.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>U.C.1.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>U.C.1.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>U.C.1.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>RoPA contains 100% of biometric and passport data processing activities as discrete entries; mismatch between RoPA and actual processing surface detected by quarterly reconciliation must close in ≤ 7 days.</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6161,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>U.C.1.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>U.C.2.1.1, U.C.2.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -6231,7 +6231,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>U.C.2.1.1, U.C.2.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -6266,7 +6266,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>U.C.2.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>U.C.2.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -6336,7 +6336,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>U.C.2.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>U.C.2.1.1, U.C.2.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>U.C.2.2.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -6441,7 +6441,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>U.C.2.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -6471,12 +6471,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-04.1-001</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>U.C.2.2.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -6491,7 +6491,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of evidence chain-of-custody records hashes match across N preservation events; 0 chain breaks in 90-day audit</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>U.C.2.3.1</t>
+          <t>UC-02</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>U.C.2.3.1</t>
+          <t>UC-02</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -6581,7 +6581,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>U.C.2.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -6616,7 +6616,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>U.C.2.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -6646,12 +6646,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-02.2-001</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>U.C.2.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>0 unsigned firmware installed in 1,000 OTA attempts; failed-signature installs blocked in ≤1s</t>
         </is>
       </c>
     </row>
@@ -6681,12 +6681,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-02.2-001</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>U.C.2.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>Rollback completes within defined RTO on 100% of failed-update drills</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>U.C.2.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>U.C.2.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -6786,12 +6786,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-02.4-001</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>U.C.2.8.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -6806,7 +6806,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>≥1 pentest report per year; 0 critical findings open &gt;30 days</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>U.C.2.3.1</t>
+          <t>UC-02</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>U.C.4.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -6891,12 +6891,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-02.1-001</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>U.C.4.2.1</t>
+          <t>UC-09</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of builds scan SCA DBs; critical CVEs block release; 0 unblocked releases in 90d</t>
         </is>
       </c>
     </row>
@@ -6931,7 +6931,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>U.C.4.3.1</t>
+          <t>UC-10</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -6961,12 +6961,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BPR-D-07.5-001</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>U.C.4.3.1</t>
+          <t>UC-10</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>100% of critical deployments carry CTO approval payload in audit log; 0 self-approved releases</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7001,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>U.C.4.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -7031,12 +7031,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-07.4-001</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>U.C.4.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of CRs have rollback plan + approver; 0 CR merges without both artefacts</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>U.C.4.2.1</t>
+          <t>UC-09</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>U.C.4.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>U.C.4.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BPR-D-07.1-002</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>U.C.4.6.1</t>
+          <t>UC-11</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of production models have version tag + rollback drill artefact; rollback restores prior accuracy within RTO</t>
         </is>
       </c>
     </row>
@@ -7211,7 +7211,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>U.C.4.3.1</t>
+          <t>UC-10</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>U.C.5.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>U.C.5.2.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -7316,7 +7316,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>U.C.5.3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -7351,7 +7351,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>U.C.5.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -7386,7 +7386,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>U.C.5.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>U.C.5.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -7451,12 +7451,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-09.3-001</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>U.C.5.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -7471,7 +7471,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>Asset inventory reconciles 100% to deployed hosts/components via nightly diff; unreconciled assets open ticket in ≤24h</t>
         </is>
       </c>
     </row>
@@ -7486,12 +7486,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-04.3-001</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>U.C.5.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -7506,7 +7506,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>100% of triggered notifications entered unified workflow; 0 missed deadlines across CRA/NIS2/GDPR/AI_Act rehearsals // HARD: provisional threshold pending multi-reg drill data</t>
         </is>
       </c>
     </row>
@@ -7521,12 +7521,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-10.2-001</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>U.C.5.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -7541,7 +7541,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of regulatory comms carry timestamp + evidence hash; 0 missing-evidence rows in 12-month report</t>
         </is>
       </c>
     </row>
@@ -7556,12 +7556,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CR-D-06.4-001</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>U.C.5.8.1</t>
+          <t>UC-12</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of cross-airport/country connections traverse isolated boundary; 0 lateral paths on purple-team test</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>U.C.5.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>U.C.6.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>U.C.6.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -7681,7 +7681,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of FR-71 (AI conformity assessment) artifacts are generated end-to-end; conformity dossier passes automated schema validation; review SLA ≤ 10 working days.</t>
         </is>
       </c>
     </row>
@@ -7701,7 +7701,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>U.C.6.2.1</t>
+          <t>UC-13</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -7731,12 +7731,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BPR-D-02.4-002</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>U.C.6.3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -7751,7 +7751,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>Quarterly bias test covers age/gender/ethnicity; ≥95% confidence interval per group; report delivered within 30d</t>
         </is>
       </c>
     </row>
@@ -7771,7 +7771,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>U.C.6.3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -7801,12 +7801,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BPR-D-10.2-002</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>U.C.6.4.1</t>
+          <t>UC-14</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of border-control decisions ship explanation payload (factors + confidence); consumer UI renders within 2s p95</t>
         </is>
       </c>
     </row>
@@ -7836,12 +7836,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BPR-D-04.5-001</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>U.C.6.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -7856,7 +7856,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>≤15 min mean detection-to-response across 50 drill runs; 0 missed critical FA/FR/drift events in 90d window // HARD: provisional threshold pending drill expansion</t>
         </is>
       </c>
     </row>
@@ -7876,7 +7876,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>U.C.6.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -7906,12 +7906,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BPR-D-02.4-001</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>U.C.6.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -7926,7 +7926,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>1 red-team/quarter; spoof-rejection rate ≥99.5% on biometric probes; report delivered within 21d</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>U.C.6.7.1</t>
+          <t>UC-15</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -7981,7 +7981,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>U.C.6.7.1</t>
+          <t>UC-15</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -8011,12 +8011,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BPR-D-10.2-002</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>U.C.6.4.1</t>
+          <t>UC-14</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>100% of FR-76 decisions have a persisted report; reports pass schema-validation; retention ≥10y</t>
         </is>
       </c>
     </row>
@@ -8051,7 +8051,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>U.C.7.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>U.C.7.2.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>U.C.7.3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -8156,7 +8156,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>U.C.7.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -8186,12 +8186,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BPR-D-08.4-001</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>U.C.7.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>≥1 quarterly simulation; click-rate trend over 4 quarters reported; high-risk users remediated ≤14d</t>
         </is>
       </c>
     </row>
@@ -8226,7 +8226,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>U.C.7.1.1, U.C.7.2.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -8422,11 +8422,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FR-28, FR-29, FR-37, FR-38, FR-39, FR-40, FR-46, FR-50, FR-52, FR-54, FR-61, FR-64</t>
+          <t>FR-28, FR-29, FR-37, FR-38, FR-39, FR-40, FR-46, FR-49, FR-50, FR-52, FR-54, FR-61, FR-64</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -8446,18 +8446,14 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-41, FR-42</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8502,18 +8498,14 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-45</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8638,11 +8630,11 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FR-21, FR-24, FR-30, FR-31, FR-34, FR-43, FR-44, FR-78</t>
+          <t>FR-21, FR-24, FR-30, FR-31, FR-34, FR-36, FR-43, FR-44, FR-78</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -8690,18 +8682,14 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-66</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -8934,18 +8922,14 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-68</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -9042,18 +9026,14 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-53</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -9202,18 +9182,14 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-65</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -9282,18 +9258,14 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-67</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9534,18 +9506,14 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-57</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -9590,18 +9558,14 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-79</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -9674,18 +9638,14 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-74</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -9842,18 +9802,14 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-77</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -9926,18 +9882,14 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-51</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -9954,18 +9906,14 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>GAP — no FR cites this rule</t>
-        </is>
-      </c>
+          <t>FR-89</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10034,7 +9982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10065,12 +10013,372 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U.C.5.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>CR-D-02.4-001, CR-D-08.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>UC-02</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CR-D-03.3-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>UC-05</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>CR-D-01.1-001, CR-D-01.2-001, CR-D-01.3-001, CR-D-01.4-001, CR-D-02.1-001, CR-D-02.2-001, CR-D-02.3-001, CR-D-02.4-001, CR-D-03.1-001, CR-D-03.2-001, CR-D-03.3-001, CR-D-03.4-001, CR-D-04.1-001, CR-D-04.2-001, CR-D-04.3-001, CR-D-04.4-001, CR-D-05.1-001, CR-D-05.2-001, CR-D-05.3-001, CR-D-05.4-001, CR-D-06.1-001, CR-D-06.2-001, CR-D-06.3-001, CR-D-06.4-001, CR-D-07.1-001, CR-D-07.2-001, CR-D-07.3-001, CR-D-07.4-001, CR-D-08.1-001, CR-D-08.2-001, CR-D-08.3-001, CR-D-09.1-001, CR-D-09.2-001, CR-D-09.3-001, CR-D-09.4-001, CR-D-10.1-001, CR-D-10.2-001, CR-D-10.3-001, BPR-D-01.1-001, BPR-D-02.1-001, BPR-D-03.1-001, BPR-D-04.5-001, BPR-D-07.1-001, BPR-D-07.5-001, BPR-D-09.1-001, BPR-D-09.5-001, BPR-D-10.4-001, BPR-D-10.5-001, BPR-D-02.4-001, BPR-D-02.4-002, BPR-D-02.5-001, BPR-D-03.1-002, BPR-D-03.5-001, BPR-D-04.2-001, BPR-D-05.1-001, BPR-D-05.5-001, BPR-D-06.5-001, BPR-D-07.1-002, BPR-D-08.4-001, BPR-D-10.2-001, BPR-D-01.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>UC-07</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CR-D-06.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UC-16</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CR-D-04.1-001, CR-D-01.1-001, BPR-D-01.1-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>UC-17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CR-D-01.2-001, CR-D-10.1-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UC-18</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CR-D-02.4-001, CR-D-10.1-001, CR-D-01.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UC-19</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CR-D-01.3-001, CR-D-10.1-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UC-20</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CR-D-01.4-001, CR-D-04.3-001, BPR-D-04.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>UC-21</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CR-D-03.2-001, CR-D-03.1-001, CR-D-10.1-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>UC-22</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CR-D-01.1-001, BPR-D-01.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>UC-23</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CR-D-10.1-001, CR-D-03.1-001, CR-D-03.2-001, CR-D-03.3-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>UC-24</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CR-D-10.1-001, CR-D-10.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UC-25</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CR-D-10.2-001, BPR-D-03.1-002, CR-D-10.1-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UC-26</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CR-D-04.1-001, CR-D-04.2-001, CR-D-10.1-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UC-27</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CR-D-10.1-001, CR-D-04.1-001, BPR-D-10.4-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UC-28</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CR-D-02.2-001, CR-D-07.3-001, CR-D-06.2-001, CR-D-01.4-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>UC-29</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CR-D-04.1-001, CR-D-04.2-001, CR-D-10.1-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>UC-30</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CR-D-04.4-001, CR-D-10.2-001, CR-D-01.1-001, CR-D-01.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UC-31</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CR-D-02.2-001, CR-D-01.4-001, CR-D-07.4-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>UC-32</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CR-D-04.2-001, CR-D-04.4-001, BPR-D-07.1-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>UC-33</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CR-D-01.1-001, CR-D-01.3-001, CR-D-05.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>UC-34</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CR-D-03.4-001, CR-D-03.3-001, CR-D-01.3-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UC-35</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CR-D-10.2-001, CR-D-10.3-001, BPR-D-10.2-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>UC-36</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CR-D-10.1-001, BPR-D-10.4-001, CR-D-10.2-001, CR-D-10.3-001, BPR-D-10.2-001, CR-D-03.4-001, CR-D-03.1-001, CR-D-01.3-001, CR-D-05.1-001, CR-D-07.1-001, CR-D-06.2-001, BPR-D-10.5-001, BPR-D-02.4-001, CR-D-03.2-001, CR-D-03.3-001, CR-D-05.4-001, CR-D-04.3-001, CR-D-09.4-001, CR-D-04.1-001, BPR-D-04.5-001, CR-D-04.2-001, BPR-D-04.2-001, CR-D-04.4-001, CR-D-02.4-001, BPR-D-02.4-002, CR-D-07.2-001, CR-D-07.4-001, BPR-D-07.1-002, CR-D-09.1-001, BPR-D-09.1-001, BPR-D-09.5-001, CR-D-09.2-001, CR-D-06.1-001, CR-D-06.3-001, BPR-D-06.5-001, CR-D-09.3-001, CR-D-08.1-001, BPR-D-08.4-001, CR-D-08.2-001, CR-D-08.3-001, CR-D-05.3-001, CR-D-02.1-001, BPR-D-02.1-001, BPR-D-02.5-001, CR-D-02.2-001, CR-D-01.1-001, BPR-D-03.1-001, BPR-D-03.5-001, BPR-D-03.1-002, CR-D-07.3-001, BPR-D-07.1-001, BPR-D-07.5-001, CR-D-06.4-001, BPR-D-05.1-001</t>
         </is>
       </c>
     </row>
@@ -12435,7 +12743,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
@@ -12518,7 +12826,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>U.C.1.2.1, U.C.3.3.1</t>
+          <t>UC-01, UC-05</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -12563,7 +12871,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -12608,7 +12916,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>U.C.2.6.1, U.C.3.3.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -12653,7 +12961,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -12698,7 +13006,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>U.C.2.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -12743,7 +13051,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -12788,7 +13096,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>U.C.6.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -12833,7 +13141,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>U.C.2.6.1, U.C.3.3.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -12878,7 +13186,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>U.C.2.1.1, U.C.2.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -12923,7 +13231,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>U.C.2.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -12968,7 +13276,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>U.C.6.4.1</t>
+          <t>UC-14</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -13013,7 +13321,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>U.C.2.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -13058,7 +13366,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>U.C.2.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -13103,7 +13411,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>U.C.4.1.1, U.C.4.3.1</t>
+          <t>UC-10</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -13148,7 +13456,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>U.C.2.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -13193,7 +13501,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>U.C.2.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -13238,7 +13546,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>U.C.2.2.1, U.C.2.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -13283,7 +13591,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -13328,7 +13636,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -13373,7 +13681,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>U.C.6.2.1</t>
+          <t>UC-13</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -13418,7 +13726,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>U.C.2.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -13463,7 +13771,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>U.C.1.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -13508,7 +13816,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>U.C.1.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -13553,7 +13861,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>U.C.1.3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -13598,7 +13906,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>U.C.1.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -13643,7 +13951,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -13688,7 +13996,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>U.C.1.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -13733,7 +14041,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>U.C.1.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -13778,7 +14086,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>U.C.1.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -13823,7 +14131,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>U.C.5.2.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -13868,7 +14176,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>U.C.2.1.1, U.C.2.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -13913,7 +14221,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>U.C.2.6.1, U.C.6.4.1</t>
+          <t>UC-14</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -13958,7 +14266,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>U.C.2.6.1, U.C.3.2.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -14003,7 +14311,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>U.C.5.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -14048,7 +14356,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>U.C.5.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -14093,7 +14401,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>U.C.2.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -14138,7 +14446,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>U.C.5.4.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -14183,7 +14491,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>U.C.5.4.1, U.C.5.7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -14228,7 +14536,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>U.C.4.5.1, U.C.5.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -14273,7 +14581,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>U.C.2.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -14318,7 +14626,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>U.C.6.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -14363,7 +14671,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>U.C.4.2.1</t>
+          <t>UC-09</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -14408,7 +14716,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>U.C.2.3.1</t>
+          <t>UC-02</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -14453,7 +14761,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>U.C.2.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -14498,7 +14806,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>U.C.6.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -14543,7 +14851,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>U.C.5.1.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -14588,7 +14896,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>U.C.6.2.1</t>
+          <t>UC-13</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -14633,7 +14941,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>U.C.6.3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -14678,7 +14986,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>U.C.6.3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -14723,7 +15031,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>U.C.6.4.1</t>
+          <t>UC-14</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -14768,7 +15076,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>U.C.3.7.1</t>
+          <t>UC-08</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -14813,7 +15121,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>U.C.6.5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -14858,7 +15166,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>U.C.4.6.1</t>
+          <t>UC-11</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -14903,7 +15211,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>U.C.6.6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -14948,7 +15256,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>U.C.6.7.1</t>
+          <t>UC-15</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -14993,7 +15301,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>U.C.6.7.1</t>
+          <t>UC-15</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">

</xml_diff>